<commit_message>
feat: strict auth hardening and optimized loading states
- Introduced AuthGate for mandatory session verification on all internal routes.
- Migrated all dashboard, admin, and operator routes to the secure /a/ prefix.
- Implemented context-aware loading: branded pulse logo is now exclusive to shop menu entries.
- Improved perceived performance with 'lite' loading for general page transitions.
- Updated all internal navigation links to match the new /a/ Account architecture.
</commit_message>
<xml_diff>
--- a/Book2.xlsx
+++ b/Book2.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="418">
   <si>
     <t>Cereals &amp; Grains</t>
   </si>
@@ -922,6 +923,363 @@
   </si>
   <si>
     <t>whey_mix.mp4</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Detox tea blends</t>
+  </si>
+  <si>
+    <t>Matcha powder</t>
+  </si>
+  <si>
+    <t>Black tea</t>
+  </si>
+  <si>
+    <t>Chamomile tea</t>
+  </si>
+  <si>
+    <t>Hibiscus tea</t>
+  </si>
+  <si>
+    <t>Green tea</t>
+  </si>
+  <si>
+    <t>Ginger tea</t>
+  </si>
+  <si>
+    <t>Lemon tea</t>
+  </si>
+  <si>
+    <t>Quinoa</t>
+  </si>
+  <si>
+    <t>Barley</t>
+  </si>
+  <si>
+    <t>Instant oats</t>
+  </si>
+  <si>
+    <t>Oats (rolled oats)</t>
+  </si>
+  <si>
+    <t>Sorghum (mtama)</t>
+  </si>
+  <si>
+    <t>Millet (wimbi)</t>
+  </si>
+  <si>
+    <t>Brown rice</t>
+  </si>
+  <si>
+    <t>Porridge flour mix</t>
+  </si>
+  <si>
+    <t>Pishori rice</t>
+  </si>
+  <si>
+    <t>Basmati rice</t>
+  </si>
+  <si>
+    <t>Granola mix</t>
+  </si>
+  <si>
+    <t>White rice</t>
+  </si>
+  <si>
+    <t>Breakfast muesli</t>
+  </si>
+  <si>
+    <t>Cornflakes</t>
+  </si>
+  <si>
+    <t>Semolina</t>
+  </si>
+  <si>
+    <t>Amaranth (terere seeds)</t>
+  </si>
+  <si>
+    <t>Wheat flour (all-purpose)</t>
+  </si>
+  <si>
+    <t>Wheat grains</t>
+  </si>
+  <si>
+    <t>Maize flour (unga ya ugali)</t>
+  </si>
+  <si>
+    <t>Maize (whole)</t>
+  </si>
+  <si>
+    <t>Olive oil</t>
+  </si>
+  <si>
+    <t>Vinegar (white)</t>
+  </si>
+  <si>
+    <t>Yeast</t>
+  </si>
+  <si>
+    <t>Baking soda</t>
+  </si>
+  <si>
+    <t>Baking powder</t>
+  </si>
+  <si>
+    <t>Soy sauce</t>
+  </si>
+  <si>
+    <t>Apple cider vinegar</t>
+  </si>
+  <si>
+    <t>Coconut oil</t>
+  </si>
+  <si>
+    <t>Cooking oil (vegetable)</t>
+  </si>
+  <si>
+    <t>Cooking oil (sunflower)</t>
+  </si>
+  <si>
+    <t>Sultanas</t>
+  </si>
+  <si>
+    <t>Raisins</t>
+  </si>
+  <si>
+    <t>Dates</t>
+  </si>
+  <si>
+    <t>Dried apricots</t>
+  </si>
+  <si>
+    <t>Dried mango</t>
+  </si>
+  <si>
+    <t>Dried pineapple</t>
+  </si>
+  <si>
+    <t>Dried bananas</t>
+  </si>
+  <si>
+    <t>Cranberries</t>
+  </si>
+  <si>
+    <t>Prunes</t>
+  </si>
+  <si>
+    <t>Date syrup</t>
+  </si>
+  <si>
+    <t>Maple syrup (imported niche)</t>
+  </si>
+  <si>
+    <t>Icing sugar</t>
+  </si>
+  <si>
+    <t>White sugar</t>
+  </si>
+  <si>
+    <t>Brown sugar</t>
+  </si>
+  <si>
+    <t>Jaggery</t>
+  </si>
+  <si>
+    <t>Molasses</t>
+  </si>
+  <si>
+    <t>Honey (processed)</t>
+  </si>
+  <si>
+    <t>Honey (raw)</t>
+  </si>
+  <si>
+    <t>Peanut butter (smooth)</t>
+  </si>
+  <si>
+    <t>Hazelnuts</t>
+  </si>
+  <si>
+    <t>Pistachios</t>
+  </si>
+  <si>
+    <t>Macadamia nuts</t>
+  </si>
+  <si>
+    <t>Walnuts</t>
+  </si>
+  <si>
+    <t>Groundnuts (roasted)</t>
+  </si>
+  <si>
+    <t>Cashew nuts</t>
+  </si>
+  <si>
+    <t>Mixed nuts pack</t>
+  </si>
+  <si>
+    <t>Groundnuts (raw)</t>
+  </si>
+  <si>
+    <t>Almond butter</t>
+  </si>
+  <si>
+    <t>Peanut butter (crunchy)</t>
+  </si>
+  <si>
+    <t>Rose coco beans</t>
+  </si>
+  <si>
+    <t>Split peas</t>
+  </si>
+  <si>
+    <t>Soya beans</t>
+  </si>
+  <si>
+    <t>Pigeon peas (mbaazi)</t>
+  </si>
+  <si>
+    <t>Cowpeas</t>
+  </si>
+  <si>
+    <t>Black beans</t>
+  </si>
+  <si>
+    <t>Lentils (green)</t>
+  </si>
+  <si>
+    <t>Lentils (red)</t>
+  </si>
+  <si>
+    <t>Chickpeas</t>
+  </si>
+  <si>
+    <t>Green grams (ndengu)</t>
+  </si>
+  <si>
+    <t>Yellow beans</t>
+  </si>
+  <si>
+    <t>Red beans</t>
+  </si>
+  <si>
+    <t>Kidney beans</t>
+  </si>
+  <si>
+    <t>Instant soup mix</t>
+  </si>
+  <si>
+    <t>Instant noodles</t>
+  </si>
+  <si>
+    <t>Breakfast biscuits</t>
+  </si>
+  <si>
+    <t>Protein bars</t>
+  </si>
+  <si>
+    <t>Energy bars</t>
+  </si>
+  <si>
+    <t>Ready porridge mix</t>
+  </si>
+  <si>
+    <t>Sunflower seeds</t>
+  </si>
+  <si>
+    <t>Flax seeds</t>
+  </si>
+  <si>
+    <t>Pumpkin seeds</t>
+  </si>
+  <si>
+    <t>Sesame seeds (white)</t>
+  </si>
+  <si>
+    <t>Hemp seeds</t>
+  </si>
+  <si>
+    <t>Poppy seeds</t>
+  </si>
+  <si>
+    <t>Basil seeds (sabja)</t>
+  </si>
+  <si>
+    <t>Mixed seed blend</t>
+  </si>
+  <si>
+    <t>Chia seeds</t>
+  </si>
+  <si>
+    <t>Sesame seeds (black)</t>
+  </si>
+  <si>
+    <t>Sea salt</t>
+  </si>
+  <si>
+    <t>Himalayan pink salt</t>
+  </si>
+  <si>
+    <t>Chili powder</t>
+  </si>
+  <si>
+    <t>Cinnamon sticks</t>
+  </si>
+  <si>
+    <t>Onion powder</t>
+  </si>
+  <si>
+    <t>Paprika</t>
+  </si>
+  <si>
+    <t>Curry powder</t>
+  </si>
+  <si>
+    <t>Turmeric powder</t>
+  </si>
+  <si>
+    <t>White pepper</t>
+  </si>
+  <si>
+    <t>Black pepper</t>
+  </si>
+  <si>
+    <t>Cayenne pepper</t>
+  </si>
+  <si>
+    <t>Ginger powder</t>
+  </si>
+  <si>
+    <t>Cinnamon powder</t>
+  </si>
+  <si>
+    <t>Cloves</t>
+  </si>
+  <si>
+    <t>Cardamom pods</t>
+  </si>
+  <si>
+    <t>Cumin seeds</t>
+  </si>
+  <si>
+    <t>Coriander seeds</t>
+  </si>
+  <si>
+    <t>Garam masala</t>
+  </si>
+  <si>
+    <t>Mixed herbs</t>
+  </si>
+  <si>
+    <t>Bay leaves</t>
+  </si>
+  <si>
+    <t>Garlic powder</t>
+  </si>
+  <si>
+    <t>Salt (table)</t>
   </si>
 </sst>
 </file>
@@ -1270,15 +1628,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AG197"/>
+  <dimension ref="A1:AK466"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="37" max="37" width="34.140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:33" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:37" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="AK1" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="C2" t="s">
         <v>152</v>
@@ -1374,72 +1738,72 @@
         <v>182</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -2160,6 +2524,1221 @@
     <row r="197" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
         <v>151</v>
+      </c>
+    </row>
+    <row r="224" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A224" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="225" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A225" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="226" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A226" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="227" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A227" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="228" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A228" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="229" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A229" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="230" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A230" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="231" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A231" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="232" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A232" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="233" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A233" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="234" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A234" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="235" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A235" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="236" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A236" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="237" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A237" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="238" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A238" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="239" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A239" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="240" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A240" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="241" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A241" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="242" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A242" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="243" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A243" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="244" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A244" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="245" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A245" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="246" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A246" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="247" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A247" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="248" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A248" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="249" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A249" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="250" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A250" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="251" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A251" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="252" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A252" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="253" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A253" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="254" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A254" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="255" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A255" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="256" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A256" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="257" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A257" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="258" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A258" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="259" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A259" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="260" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A260" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="261" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A261" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="262" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A262" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="263" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A263" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="264" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A264" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="265" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A265" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="266" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A266" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="267" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A267" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="268" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A268" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="269" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A269" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="270" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A270" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="271" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A271" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="272" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A272" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="273" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A273" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="274" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A274" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="275" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A275" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="276" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A276" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="277" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A277" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="278" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A278" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="279" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A279" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="280" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A280" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="281" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A281" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="282" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A282" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="283" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A283" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="284" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A284" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="285" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A285" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="286" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A286" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="287" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A287" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="288" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A288" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="289" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A289" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="290" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A290" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="291" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A291" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="292" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A292" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="293" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A293" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="294" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A294" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="295" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A295" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="296" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A296" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="297" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A297" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="298" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A298" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="299" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A299" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="300" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A300" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="301" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A301" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="302" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A302" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="303" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A303" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="304" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A304" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="305" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A305" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="306" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A306" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="307" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A307" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="308" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A308" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="309" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A309" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="310" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A310" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="311" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A311" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="312" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A312" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="313" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A313" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="314" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A314" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="315" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A315" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="316" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A316" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="317" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A317" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="318" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A318" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="319" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A319" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="320" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A320" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="321" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A321" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="322" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A322" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="323" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A323" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="324" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A324" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="325" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A325" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="326" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A326" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="327" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A327" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="328" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A328" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="329" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A329" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="330" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A330" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="331" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A331" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="332" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A332" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="333" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A333" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="334" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A334" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="335" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A335" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="336" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A336" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="337" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A337" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="338" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A338" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="339" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A339" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="340" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A340" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="341" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A341" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="342" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A342" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="343" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A343" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="344" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A344" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="345" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A345" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="346" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A346" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="347" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A347" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="348" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A348" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="349" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A349" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="350" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A350" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="351" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A351" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="352" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A352" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="353" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A353" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="354" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A354" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="355" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A355" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="356" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A356" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="357" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A357" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="358" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A358" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="359" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A359" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="360" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A360" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="361" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A361" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="362" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A362" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="363" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A363" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="364" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A364" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="365" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A365" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="366" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A366" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="367" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A367" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="368" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A368" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="369" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A369" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="370" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A370" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="371" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A371" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="372" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A372" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="373" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A373" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="374" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A374" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="375" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A375" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="376" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A376" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="377" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A377" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="378" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A378" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="379" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A379" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="380" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A380" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="381" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A381" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="382" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A382" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="383" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A383" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="384" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A384" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="385" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A385" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="386" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A386" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="387" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A387" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="388" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A388" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="389" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A389" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="390" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A390" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="391" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A391" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="392" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A392" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="393" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A393" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="394" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A394" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="395" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A395" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="396" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A396" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="397" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A397" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="398" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A398" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="399" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A399" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="400" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A400" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="401" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A401" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="402" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A402" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="403" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A403" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="404" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A404" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="405" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A405" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="406" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A406" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="407" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A407" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="408" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A408" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="409" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A409" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="410" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A410" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="411" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A411" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="412" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A412" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="413" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A413" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="414" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A414" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="415" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A415" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="416" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A416" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="417" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A417" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="418" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A418" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="419" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A419" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="420" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A420" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="421" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A421" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="422" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A422" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="423" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A423" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="424" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A424" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="425" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A425" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="426" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A426" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="427" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A427" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="428" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A428" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="429" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A429" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="430" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A430" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="431" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A431" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="432" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A432" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="433" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A433" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="434" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A434" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="435" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A435" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="436" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A436" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="437" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A437" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="438" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A438" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="439" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A439" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="440" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A440" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="441" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A441" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="442" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A442" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="443" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A443" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="444" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A444" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="445" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A445" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="446" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A446" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="447" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A447" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="448" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A448" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="449" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A449" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="450" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A450" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="451" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A451" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="452" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A452" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="453" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A453" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="454" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A454" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="455" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A455" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="456" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A456" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="457" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A457" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="458" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A458" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="459" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A459" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="460" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A460" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="461" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A461" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="462" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A462" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="463" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A463" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="464" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A464" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="465" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A465" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="466" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A466" t="s">
+        <v>284</v>
       </c>
     </row>
   </sheetData>
@@ -2171,6 +3750,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Y6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.42578125" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="16.5703125" customWidth="1"/>
+    <col min="9" max="9" width="15.28515625" customWidth="1"/>
+    <col min="10" max="10" width="15.5703125" customWidth="1"/>
+    <col min="11" max="11" width="13.5703125" customWidth="1"/>
+    <col min="12" max="12" width="17.140625" customWidth="1"/>
+    <col min="13" max="13" width="20" customWidth="1"/>
+    <col min="14" max="14" width="19.85546875" customWidth="1"/>
+    <col min="15" max="15" width="16.7109375" customWidth="1"/>
+    <col min="16" max="16" width="16.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">

</xml_diff>